<commit_message>
evoluindo a engenharia de colunas
</commit_message>
<xml_diff>
--- a/Dados/Modelo ERD e Tabelas de Apoio.xlsx
+++ b/Dados/Modelo ERD e Tabelas de Apoio.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kaue Mandarino\Desktop\Mestrado\degrees\Projeto-Turin\Dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE377F57-11C3-4423-A711-BF29065F7735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3FDAECF-EB25-4907-B220-E6C6DA93DD7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{AD869555-1455-4E4D-8A0B-B7149227DFB8}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1590" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1591" uniqueCount="278">
   <si>
     <t>dim_obitos</t>
   </si>
@@ -879,13 +879,16 @@
   </si>
   <si>
     <t>Natal</t>
+  </si>
+  <si>
+    <t>nome_uf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -933,6 +936,13 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF00B050"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFF00"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1172,7 +1182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1314,6 +1324,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -11317,10 +11330,10 @@
       <c r="B8" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="48" t="s">
+      <c r="C8" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="48" t="s">
+      <c r="D8" s="49" t="s">
         <v>148</v>
       </c>
       <c r="G8" s="5" t="s">
@@ -11328,10 +11341,10 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="48" t="s">
         <v>150</v>
       </c>
       <c r="G9" s="5" t="s">
@@ -11806,8 +11819,8 @@
       <c r="A22" s="38" t="s">
         <v>72</v>
       </c>
-      <c r="B22" s="39">
-        <v>1</v>
+      <c r="B22" s="39" t="s">
+        <v>277</v>
       </c>
       <c r="C22" s="40" t="s">
         <v>73</v>

</xml_diff>